<commit_message>
update teitle dan subtitle modal edit dan tambah
</commit_message>
<xml_diff>
--- a/database/seeders/data/data_mapel.xlsx
+++ b/database/seeders/data/data_mapel.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BAHASA_PEROGRAMAN\LARAVEL\simantab\database\seeders\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3191DD-97C4-4770-A1C4-6587955D2818}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{012DBBC3-3E7B-4947-82A8-CA9CA80129DE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{16929766-A6C7-49F7-8F1B-817CC57C92D2}"/>
   </bookViews>
@@ -1239,9 +1239,6 @@
     <t>SD</t>
   </si>
   <si>
-    <t>KURMER-2026-2027</t>
-  </si>
-  <si>
     <t>kode_kurikulum</t>
   </si>
   <si>
@@ -1273,6 +1270,9 @@
   </si>
   <si>
     <t>PAKET-C</t>
+  </si>
+  <si>
+    <t>KKM002</t>
   </si>
 </sst>
 </file>
@@ -1650,10 +1650,10 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
+        <v>403</v>
+      </c>
+      <c r="E1" t="s">
         <v>404</v>
-      </c>
-      <c r="E1" t="s">
-        <v>405</v>
       </c>
       <c r="F1" t="s">
         <v>2</v>
@@ -1673,7 +1673,7 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E2" t="s">
         <v>401</v>
@@ -1696,7 +1696,7 @@
         <v>75</v>
       </c>
       <c r="D3" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E3" t="s">
         <v>401</v>
@@ -1719,7 +1719,7 @@
         <v>75</v>
       </c>
       <c r="D4" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E4" t="s">
         <v>401</v>
@@ -1742,7 +1742,7 @@
         <v>75</v>
       </c>
       <c r="D5" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E5" t="s">
         <v>402</v>
@@ -1765,7 +1765,7 @@
         <v>75</v>
       </c>
       <c r="D6" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E6" t="s">
         <v>402</v>
@@ -1788,7 +1788,7 @@
         <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E7" t="s">
         <v>402</v>
@@ -1811,7 +1811,7 @@
         <v>75</v>
       </c>
       <c r="D8" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E8" t="s">
         <v>402</v>
@@ -1834,7 +1834,7 @@
         <v>75</v>
       </c>
       <c r="D9" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E9" t="s">
         <v>402</v>
@@ -1857,7 +1857,7 @@
         <v>75</v>
       </c>
       <c r="D10" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E10" t="s">
         <v>402</v>
@@ -1880,7 +1880,7 @@
         <v>75</v>
       </c>
       <c r="D11" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E11" t="s">
         <v>402</v>
@@ -1903,7 +1903,7 @@
         <v>75</v>
       </c>
       <c r="D12" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E12" t="s">
         <v>402</v>
@@ -1926,7 +1926,7 @@
         <v>75</v>
       </c>
       <c r="D13" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E13" t="s">
         <v>402</v>
@@ -1949,7 +1949,7 @@
         <v>75</v>
       </c>
       <c r="D14" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E14" t="s">
         <v>402</v>
@@ -1972,7 +1972,7 @@
         <v>75</v>
       </c>
       <c r="D15" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E15" t="s">
         <v>402</v>
@@ -1995,7 +1995,7 @@
         <v>75</v>
       </c>
       <c r="D16" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E16" t="s">
         <v>402</v>
@@ -2018,7 +2018,7 @@
         <v>75</v>
       </c>
       <c r="D17" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E17" t="s">
         <v>402</v>
@@ -2041,7 +2041,7 @@
         <v>75</v>
       </c>
       <c r="D18" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E18" t="s">
         <v>402</v>
@@ -2064,7 +2064,7 @@
         <v>75</v>
       </c>
       <c r="D19" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E19" t="s">
         <v>402</v>
@@ -2087,7 +2087,7 @@
         <v>75</v>
       </c>
       <c r="D20" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E20" t="s">
         <v>402</v>
@@ -2110,7 +2110,7 @@
         <v>75</v>
       </c>
       <c r="D21" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E21" t="s">
         <v>402</v>
@@ -2133,7 +2133,7 @@
         <v>75</v>
       </c>
       <c r="D22" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E22" t="s">
         <v>402</v>
@@ -2156,7 +2156,7 @@
         <v>75</v>
       </c>
       <c r="D23" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E23" t="s">
         <v>402</v>
@@ -2179,7 +2179,7 @@
         <v>75</v>
       </c>
       <c r="D24" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E24" t="s">
         <v>402</v>
@@ -2202,7 +2202,7 @@
         <v>75</v>
       </c>
       <c r="D25" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E25" t="s">
         <v>402</v>
@@ -2225,7 +2225,7 @@
         <v>75</v>
       </c>
       <c r="D26" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E26" t="s">
         <v>402</v>
@@ -2248,7 +2248,7 @@
         <v>75</v>
       </c>
       <c r="D27" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E27" t="s">
         <v>402</v>
@@ -2271,7 +2271,7 @@
         <v>75</v>
       </c>
       <c r="D28" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E28" t="s">
         <v>402</v>
@@ -2294,7 +2294,7 @@
         <v>75</v>
       </c>
       <c r="D29" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E29" t="s">
         <v>402</v>
@@ -2317,7 +2317,7 @@
         <v>75</v>
       </c>
       <c r="D30" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E30" t="s">
         <v>402</v>
@@ -2340,10 +2340,10 @@
         <v>75</v>
       </c>
       <c r="D31" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E31" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F31" t="s">
         <v>7</v>
@@ -2363,10 +2363,10 @@
         <v>75</v>
       </c>
       <c r="D32" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E32" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F32" t="s">
         <v>7</v>
@@ -2386,10 +2386,10 @@
         <v>75</v>
       </c>
       <c r="D33" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E33" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F33" t="s">
         <v>7</v>
@@ -2409,10 +2409,10 @@
         <v>75</v>
       </c>
       <c r="D34" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E34" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F34" t="s">
         <v>7</v>
@@ -2432,10 +2432,10 @@
         <v>75</v>
       </c>
       <c r="D35" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E35" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F35" t="s">
         <v>7</v>
@@ -2455,10 +2455,10 @@
         <v>75</v>
       </c>
       <c r="D36" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E36" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F36" t="s">
         <v>7</v>
@@ -2478,10 +2478,10 @@
         <v>75</v>
       </c>
       <c r="D37" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E37" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F37" t="s">
         <v>7</v>
@@ -2501,10 +2501,10 @@
         <v>75</v>
       </c>
       <c r="D38" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E38" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F38" t="s">
         <v>7</v>
@@ -2524,10 +2524,10 @@
         <v>75</v>
       </c>
       <c r="D39" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E39" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F39" t="s">
         <v>7</v>
@@ -2547,10 +2547,10 @@
         <v>75</v>
       </c>
       <c r="D40" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E40" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F40" t="s">
         <v>7</v>
@@ -2570,10 +2570,10 @@
         <v>75</v>
       </c>
       <c r="D41" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E41" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F41" t="s">
         <v>7</v>
@@ -2593,10 +2593,10 @@
         <v>75</v>
       </c>
       <c r="D42" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E42" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F42" t="s">
         <v>7</v>
@@ -2616,10 +2616,10 @@
         <v>75</v>
       </c>
       <c r="D43" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E43" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F43" t="s">
         <v>7</v>
@@ -2639,10 +2639,10 @@
         <v>75</v>
       </c>
       <c r="D44" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E44" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F44" t="s">
         <v>7</v>
@@ -2662,10 +2662,10 @@
         <v>75</v>
       </c>
       <c r="D45" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E45" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F45" t="s">
         <v>7</v>
@@ -2685,10 +2685,10 @@
         <v>75</v>
       </c>
       <c r="D46" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E46" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F46" t="s">
         <v>52</v>
@@ -2708,10 +2708,10 @@
         <v>75</v>
       </c>
       <c r="D47" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E47" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="F47" t="s">
         <v>55</v>
@@ -2731,10 +2731,10 @@
         <v>75</v>
       </c>
       <c r="D48" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E48" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F48" t="s">
         <v>7</v>
@@ -2754,10 +2754,10 @@
         <v>75</v>
       </c>
       <c r="D49" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E49" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F49" t="s">
         <v>7</v>
@@ -2777,10 +2777,10 @@
         <v>75</v>
       </c>
       <c r="D50" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E50" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F50" t="s">
         <v>7</v>
@@ -2800,10 +2800,10 @@
         <v>75</v>
       </c>
       <c r="D51" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E51" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F51" t="s">
         <v>7</v>
@@ -2823,10 +2823,10 @@
         <v>75</v>
       </c>
       <c r="D52" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E52" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F52" t="s">
         <v>7</v>
@@ -2846,10 +2846,10 @@
         <v>75</v>
       </c>
       <c r="D53" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E53" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F53" t="s">
         <v>7</v>
@@ -2869,10 +2869,10 @@
         <v>75</v>
       </c>
       <c r="D54" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E54" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F54" t="s">
         <v>7</v>
@@ -2892,10 +2892,10 @@
         <v>75</v>
       </c>
       <c r="D55" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E55" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F55" t="s">
         <v>7</v>
@@ -2915,10 +2915,10 @@
         <v>75</v>
       </c>
       <c r="D56" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E56" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F56" t="s">
         <v>7</v>
@@ -2938,10 +2938,10 @@
         <v>75</v>
       </c>
       <c r="D57" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E57" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F57" t="s">
         <v>7</v>
@@ -2961,10 +2961,10 @@
         <v>75</v>
       </c>
       <c r="D58" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E58" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F58" t="s">
         <v>7</v>
@@ -2984,10 +2984,10 @@
         <v>75</v>
       </c>
       <c r="D59" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E59" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F59" t="s">
         <v>7</v>
@@ -3007,10 +3007,10 @@
         <v>75</v>
       </c>
       <c r="D60" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E60" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F60" t="s">
         <v>7</v>
@@ -3030,10 +3030,10 @@
         <v>75</v>
       </c>
       <c r="D61" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E61" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F61" t="s">
         <v>7</v>
@@ -3053,10 +3053,10 @@
         <v>75</v>
       </c>
       <c r="D62" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E62" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F62" t="s">
         <v>7</v>
@@ -3076,10 +3076,10 @@
         <v>75</v>
       </c>
       <c r="D63" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E63" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F63" t="s">
         <v>52</v>
@@ -3099,10 +3099,10 @@
         <v>75</v>
       </c>
       <c r="D64" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E64" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F64" t="s">
         <v>55</v>
@@ -3122,10 +3122,10 @@
         <v>75</v>
       </c>
       <c r="D65" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E65" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F65" t="s">
         <v>7</v>
@@ -3145,10 +3145,10 @@
         <v>75</v>
       </c>
       <c r="D66" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E66" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F66" t="s">
         <v>7</v>
@@ -3168,10 +3168,10 @@
         <v>75</v>
       </c>
       <c r="D67" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E67" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F67" t="s">
         <v>7</v>
@@ -3191,10 +3191,10 @@
         <v>75</v>
       </c>
       <c r="D68" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E68" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F68" t="s">
         <v>7</v>
@@ -3214,10 +3214,10 @@
         <v>75</v>
       </c>
       <c r="D69" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E69" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F69" t="s">
         <v>7</v>
@@ -3237,10 +3237,10 @@
         <v>75</v>
       </c>
       <c r="D70" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E70" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F70" t="s">
         <v>7</v>
@@ -3260,10 +3260,10 @@
         <v>75</v>
       </c>
       <c r="D71" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E71" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F71" t="s">
         <v>7</v>
@@ -3283,10 +3283,10 @@
         <v>75</v>
       </c>
       <c r="D72" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E72" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F72" t="s">
         <v>7</v>
@@ -3306,10 +3306,10 @@
         <v>75</v>
       </c>
       <c r="D73" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E73" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F73" t="s">
         <v>7</v>
@@ -3329,10 +3329,10 @@
         <v>75</v>
       </c>
       <c r="D74" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E74" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F74" t="s">
         <v>7</v>
@@ -3352,10 +3352,10 @@
         <v>75</v>
       </c>
       <c r="D75" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E75" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F75" t="s">
         <v>7</v>
@@ -3375,10 +3375,10 @@
         <v>75</v>
       </c>
       <c r="D76" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E76" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F76" t="s">
         <v>7</v>
@@ -3398,10 +3398,10 @@
         <v>75</v>
       </c>
       <c r="D77" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E77" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F77" t="s">
         <v>7</v>
@@ -3421,10 +3421,10 @@
         <v>75</v>
       </c>
       <c r="D78" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E78" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F78" t="s">
         <v>52</v>
@@ -3444,10 +3444,10 @@
         <v>75</v>
       </c>
       <c r="D79" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E79" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F79" t="s">
         <v>52</v>
@@ -3467,10 +3467,10 @@
         <v>75</v>
       </c>
       <c r="D80" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E80" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F80" t="s">
         <v>52</v>
@@ -3490,10 +3490,10 @@
         <v>75</v>
       </c>
       <c r="D81" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E81" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F81" t="s">
         <v>52</v>
@@ -3513,10 +3513,10 @@
         <v>75</v>
       </c>
       <c r="D82" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E82" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F82" t="s">
         <v>52</v>
@@ -3536,10 +3536,10 @@
         <v>75</v>
       </c>
       <c r="D83" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E83" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F83" t="s">
         <v>52</v>
@@ -3559,10 +3559,10 @@
         <v>75</v>
       </c>
       <c r="D84" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E84" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F84" t="s">
         <v>52</v>
@@ -3582,10 +3582,10 @@
         <v>75</v>
       </c>
       <c r="D85" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E85" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F85" t="s">
         <v>52</v>
@@ -3605,10 +3605,10 @@
         <v>75</v>
       </c>
       <c r="D86" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E86" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F86" t="s">
         <v>52</v>
@@ -3628,10 +3628,10 @@
         <v>75</v>
       </c>
       <c r="D87" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E87" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F87" t="s">
         <v>52</v>
@@ -3651,10 +3651,10 @@
         <v>75</v>
       </c>
       <c r="D88" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E88" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F88" t="s">
         <v>52</v>
@@ -3674,10 +3674,10 @@
         <v>75</v>
       </c>
       <c r="D89" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E89" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F89" t="s">
         <v>52</v>
@@ -3697,10 +3697,10 @@
         <v>75</v>
       </c>
       <c r="D90" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E90" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F90" t="s">
         <v>52</v>
@@ -3720,10 +3720,10 @@
         <v>75</v>
       </c>
       <c r="D91" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E91" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F91" t="s">
         <v>52</v>
@@ -3743,10 +3743,10 @@
         <v>75</v>
       </c>
       <c r="D92" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E92" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F92" t="s">
         <v>52</v>
@@ -3766,10 +3766,10 @@
         <v>75</v>
       </c>
       <c r="D93" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E93" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F93" t="s">
         <v>52</v>
@@ -3789,10 +3789,10 @@
         <v>75</v>
       </c>
       <c r="D94" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E94" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F94" t="s">
         <v>52</v>
@@ -3812,10 +3812,10 @@
         <v>75</v>
       </c>
       <c r="D95" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E95" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F95" t="s">
         <v>52</v>
@@ -3835,10 +3835,10 @@
         <v>75</v>
       </c>
       <c r="D96" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E96" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F96" t="s">
         <v>52</v>
@@ -3858,10 +3858,10 @@
         <v>75</v>
       </c>
       <c r="D97" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E97" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F97" t="s">
         <v>52</v>
@@ -3881,10 +3881,10 @@
         <v>75</v>
       </c>
       <c r="D98" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E98" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="F98" t="s">
         <v>55</v>
@@ -3904,10 +3904,10 @@
         <v>75</v>
       </c>
       <c r="D99" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E99" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F99" t="s">
         <v>7</v>
@@ -3927,10 +3927,10 @@
         <v>75</v>
       </c>
       <c r="D100" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E100" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F100" t="s">
         <v>7</v>
@@ -3950,10 +3950,10 @@
         <v>75</v>
       </c>
       <c r="D101" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E101" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F101" t="s">
         <v>7</v>
@@ -3973,10 +3973,10 @@
         <v>75</v>
       </c>
       <c r="D102" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E102" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F102" t="s">
         <v>7</v>
@@ -3996,10 +3996,10 @@
         <v>75</v>
       </c>
       <c r="D103" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E103" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F103" t="s">
         <v>7</v>
@@ -4019,10 +4019,10 @@
         <v>75</v>
       </c>
       <c r="D104" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E104" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F104" t="s">
         <v>7</v>
@@ -4042,10 +4042,10 @@
         <v>75</v>
       </c>
       <c r="D105" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E105" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F105" t="s">
         <v>7</v>
@@ -4065,10 +4065,10 @@
         <v>75</v>
       </c>
       <c r="D106" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E106" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F106" t="s">
         <v>7</v>
@@ -4088,10 +4088,10 @@
         <v>75</v>
       </c>
       <c r="D107" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E107" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F107" t="s">
         <v>7</v>
@@ -4111,10 +4111,10 @@
         <v>75</v>
       </c>
       <c r="D108" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E108" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F108" t="s">
         <v>7</v>
@@ -4134,10 +4134,10 @@
         <v>75</v>
       </c>
       <c r="D109" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E109" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F109" t="s">
         <v>7</v>
@@ -4157,10 +4157,10 @@
         <v>75</v>
       </c>
       <c r="D110" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E110" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F110" t="s">
         <v>7</v>
@@ -4180,10 +4180,10 @@
         <v>75</v>
       </c>
       <c r="D111" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E111" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F111" t="s">
         <v>7</v>
@@ -4203,10 +4203,10 @@
         <v>75</v>
       </c>
       <c r="D112" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E112" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F112" t="s">
         <v>7</v>
@@ -4226,10 +4226,10 @@
         <v>75</v>
       </c>
       <c r="D113" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E113" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F113" t="s">
         <v>7</v>
@@ -4249,10 +4249,10 @@
         <v>75</v>
       </c>
       <c r="D114" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E114" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F114" t="s">
         <v>7</v>
@@ -4272,10 +4272,10 @@
         <v>75</v>
       </c>
       <c r="D115" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E115" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F115" t="s">
         <v>52</v>
@@ -4295,10 +4295,10 @@
         <v>75</v>
       </c>
       <c r="D116" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E116" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F116" t="s">
         <v>55</v>
@@ -4318,10 +4318,10 @@
         <v>75</v>
       </c>
       <c r="D117" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E117" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F117" t="s">
         <v>7</v>
@@ -4341,10 +4341,10 @@
         <v>75</v>
       </c>
       <c r="D118" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E118" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F118" t="s">
         <v>7</v>
@@ -4364,10 +4364,10 @@
         <v>75</v>
       </c>
       <c r="D119" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E119" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F119" t="s">
         <v>7</v>
@@ -4387,10 +4387,10 @@
         <v>75</v>
       </c>
       <c r="D120" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E120" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F120" t="s">
         <v>7</v>
@@ -4410,10 +4410,10 @@
         <v>75</v>
       </c>
       <c r="D121" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E121" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F121" t="s">
         <v>7</v>
@@ -4433,10 +4433,10 @@
         <v>75</v>
       </c>
       <c r="D122" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E122" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F122" t="s">
         <v>7</v>
@@ -4456,10 +4456,10 @@
         <v>75</v>
       </c>
       <c r="D123" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E123" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F123" t="s">
         <v>7</v>
@@ -4479,10 +4479,10 @@
         <v>75</v>
       </c>
       <c r="D124" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E124" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F124" t="s">
         <v>7</v>
@@ -4502,10 +4502,10 @@
         <v>75</v>
       </c>
       <c r="D125" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E125" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F125" t="s">
         <v>7</v>
@@ -4525,10 +4525,10 @@
         <v>75</v>
       </c>
       <c r="D126" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E126" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F126" t="s">
         <v>7</v>
@@ -4548,10 +4548,10 @@
         <v>75</v>
       </c>
       <c r="D127" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E127" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F127" t="s">
         <v>7</v>
@@ -4571,10 +4571,10 @@
         <v>75</v>
       </c>
       <c r="D128" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E128" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F128" t="s">
         <v>52</v>
@@ -4594,10 +4594,10 @@
         <v>75</v>
       </c>
       <c r="D129" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E129" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F129" t="s">
         <v>52</v>
@@ -4617,10 +4617,10 @@
         <v>75</v>
       </c>
       <c r="D130" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E130" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F130" t="s">
         <v>52</v>
@@ -4640,10 +4640,10 @@
         <v>75</v>
       </c>
       <c r="D131" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E131" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F131" t="s">
         <v>52</v>
@@ -4663,10 +4663,10 @@
         <v>75</v>
       </c>
       <c r="D132" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E132" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F132" t="s">
         <v>52</v>
@@ -4686,10 +4686,10 @@
         <v>75</v>
       </c>
       <c r="D133" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E133" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F133" t="s">
         <v>55</v>
@@ -4709,10 +4709,10 @@
         <v>75</v>
       </c>
       <c r="D134" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E134" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F134" t="s">
         <v>52</v>
@@ -4732,10 +4732,10 @@
         <v>75</v>
       </c>
       <c r="D135" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E135" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F135" t="s">
         <v>52</v>
@@ -4755,10 +4755,10 @@
         <v>75</v>
       </c>
       <c r="D136" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E136" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F136" t="s">
         <v>52</v>
@@ -4778,10 +4778,10 @@
         <v>75</v>
       </c>
       <c r="D137" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E137" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F137" t="s">
         <v>52</v>
@@ -4801,10 +4801,10 @@
         <v>75</v>
       </c>
       <c r="D138" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E138" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F138" t="s">
         <v>52</v>
@@ -4824,10 +4824,10 @@
         <v>75</v>
       </c>
       <c r="D139" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E139" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="F139" t="s">
         <v>55</v>
@@ -4847,10 +4847,10 @@
         <v>75</v>
       </c>
       <c r="D140" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E140" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F140" t="s">
         <v>7</v>
@@ -4870,10 +4870,10 @@
         <v>75</v>
       </c>
       <c r="D141" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E141" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F141" t="s">
         <v>7</v>
@@ -4893,10 +4893,10 @@
         <v>75</v>
       </c>
       <c r="D142" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E142" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F142" t="s">
         <v>7</v>
@@ -4916,10 +4916,10 @@
         <v>75</v>
       </c>
       <c r="D143" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E143" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F143" t="s">
         <v>7</v>
@@ -4939,10 +4939,10 @@
         <v>75</v>
       </c>
       <c r="D144" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E144" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F144" t="s">
         <v>7</v>
@@ -4962,10 +4962,10 @@
         <v>75</v>
       </c>
       <c r="D145" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E145" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F145" t="s">
         <v>7</v>
@@ -4985,10 +4985,10 @@
         <v>75</v>
       </c>
       <c r="D146" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E146" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F146" t="s">
         <v>7</v>
@@ -5008,10 +5008,10 @@
         <v>75</v>
       </c>
       <c r="D147" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E147" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F147" t="s">
         <v>7</v>
@@ -5031,10 +5031,10 @@
         <v>75</v>
       </c>
       <c r="D148" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E148" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F148" t="s">
         <v>7</v>
@@ -5054,10 +5054,10 @@
         <v>75</v>
       </c>
       <c r="D149" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E149" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F149" t="s">
         <v>7</v>
@@ -5077,10 +5077,10 @@
         <v>75</v>
       </c>
       <c r="D150" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E150" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F150" t="s">
         <v>7</v>
@@ -5100,10 +5100,10 @@
         <v>75</v>
       </c>
       <c r="D151" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E151" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F151" t="s">
         <v>7</v>
@@ -5123,10 +5123,10 @@
         <v>75</v>
       </c>
       <c r="D152" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E152" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F152" t="s">
         <v>7</v>
@@ -5146,10 +5146,10 @@
         <v>75</v>
       </c>
       <c r="D153" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E153" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F153" t="s">
         <v>214</v>
@@ -5169,10 +5169,10 @@
         <v>75</v>
       </c>
       <c r="D154" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E154" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F154" t="s">
         <v>214</v>
@@ -5192,10 +5192,10 @@
         <v>75</v>
       </c>
       <c r="D155" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E155" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F155" t="s">
         <v>214</v>
@@ -5215,10 +5215,10 @@
         <v>75</v>
       </c>
       <c r="D156" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E156" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F156" t="s">
         <v>214</v>
@@ -5238,10 +5238,10 @@
         <v>75</v>
       </c>
       <c r="D157" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E157" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F157" t="s">
         <v>214</v>
@@ -5261,10 +5261,10 @@
         <v>75</v>
       </c>
       <c r="D158" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E158" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="F158" t="s">
         <v>55</v>
@@ -5284,10 +5284,10 @@
         <v>75</v>
       </c>
       <c r="D159" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E159" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F159" t="s">
         <v>7</v>
@@ -5307,10 +5307,10 @@
         <v>75</v>
       </c>
       <c r="D160" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E160" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F160" t="s">
         <v>7</v>
@@ -5330,10 +5330,10 @@
         <v>75</v>
       </c>
       <c r="D161" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E161" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F161" t="s">
         <v>7</v>
@@ -5353,10 +5353,10 @@
         <v>75</v>
       </c>
       <c r="D162" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E162" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F162" t="s">
         <v>7</v>
@@ -5376,10 +5376,10 @@
         <v>75</v>
       </c>
       <c r="D163" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E163" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F163" t="s">
         <v>7</v>
@@ -5399,10 +5399,10 @@
         <v>75</v>
       </c>
       <c r="D164" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E164" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F164" t="s">
         <v>7</v>
@@ -5422,10 +5422,10 @@
         <v>75</v>
       </c>
       <c r="D165" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E165" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F165" t="s">
         <v>7</v>
@@ -5445,10 +5445,10 @@
         <v>75</v>
       </c>
       <c r="D166" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E166" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F166" t="s">
         <v>7</v>
@@ -5468,10 +5468,10 @@
         <v>75</v>
       </c>
       <c r="D167" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E167" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F167" t="s">
         <v>7</v>
@@ -5491,10 +5491,10 @@
         <v>75</v>
       </c>
       <c r="D168" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E168" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F168" t="s">
         <v>7</v>
@@ -5514,10 +5514,10 @@
         <v>75</v>
       </c>
       <c r="D169" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E169" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F169" t="s">
         <v>7</v>
@@ -5537,10 +5537,10 @@
         <v>75</v>
       </c>
       <c r="D170" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E170" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F170" t="s">
         <v>7</v>
@@ -5560,10 +5560,10 @@
         <v>75</v>
       </c>
       <c r="D171" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E171" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F171" t="s">
         <v>7</v>
@@ -5583,10 +5583,10 @@
         <v>75</v>
       </c>
       <c r="D172" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E172" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F172" t="s">
         <v>7</v>
@@ -5606,10 +5606,10 @@
         <v>75</v>
       </c>
       <c r="D173" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E173" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F173" t="s">
         <v>240</v>
@@ -5629,10 +5629,10 @@
         <v>75</v>
       </c>
       <c r="D174" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E174" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F174" t="s">
         <v>240</v>
@@ -5652,10 +5652,10 @@
         <v>75</v>
       </c>
       <c r="D175" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E175" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F175" t="s">
         <v>240</v>
@@ -5675,10 +5675,10 @@
         <v>75</v>
       </c>
       <c r="D176" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E176" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F176" t="s">
         <v>240</v>
@@ -5698,10 +5698,10 @@
         <v>75</v>
       </c>
       <c r="D177" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E177" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F177" t="s">
         <v>240</v>
@@ -5721,10 +5721,10 @@
         <v>75</v>
       </c>
       <c r="D178" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E178" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F178" t="s">
         <v>240</v>
@@ -5744,10 +5744,10 @@
         <v>75</v>
       </c>
       <c r="D179" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E179" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F179" t="s">
         <v>240</v>
@@ -5767,10 +5767,10 @@
         <v>75</v>
       </c>
       <c r="D180" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E180" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F180" t="s">
         <v>240</v>
@@ -5790,10 +5790,10 @@
         <v>75</v>
       </c>
       <c r="D181" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E181" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F181" t="s">
         <v>240</v>
@@ -5813,10 +5813,10 @@
         <v>75</v>
       </c>
       <c r="D182" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E182" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F182" t="s">
         <v>240</v>
@@ -5836,10 +5836,10 @@
         <v>75</v>
       </c>
       <c r="D183" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E183" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F183" t="s">
         <v>240</v>
@@ -5859,10 +5859,10 @@
         <v>75</v>
       </c>
       <c r="D184" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E184" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F184" t="s">
         <v>240</v>
@@ -5882,10 +5882,10 @@
         <v>75</v>
       </c>
       <c r="D185" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E185" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F185" t="s">
         <v>240</v>
@@ -5905,10 +5905,10 @@
         <v>75</v>
       </c>
       <c r="D186" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E186" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F186" t="s">
         <v>240</v>
@@ -5928,10 +5928,10 @@
         <v>75</v>
       </c>
       <c r="D187" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E187" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F187" t="s">
         <v>240</v>
@@ -5951,10 +5951,10 @@
         <v>75</v>
       </c>
       <c r="D188" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E188" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F188" t="s">
         <v>240</v>
@@ -5974,10 +5974,10 @@
         <v>75</v>
       </c>
       <c r="D189" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E189" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F189" t="s">
         <v>240</v>
@@ -5997,10 +5997,10 @@
         <v>75</v>
       </c>
       <c r="D190" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E190" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F190" t="s">
         <v>240</v>
@@ -6020,10 +6020,10 @@
         <v>75</v>
       </c>
       <c r="D191" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E191" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F191" t="s">
         <v>240</v>
@@ -6043,10 +6043,10 @@
         <v>75</v>
       </c>
       <c r="D192" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E192" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F192" t="s">
         <v>240</v>
@@ -6066,10 +6066,10 @@
         <v>75</v>
       </c>
       <c r="D193" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E193" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F193" t="s">
         <v>240</v>
@@ -6089,10 +6089,10 @@
         <v>75</v>
       </c>
       <c r="D194" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E194" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F194" t="s">
         <v>214</v>
@@ -6112,10 +6112,10 @@
         <v>75</v>
       </c>
       <c r="D195" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E195" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F195" t="s">
         <v>214</v>
@@ -6135,10 +6135,10 @@
         <v>75</v>
       </c>
       <c r="D196" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E196" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F196" t="s">
         <v>214</v>
@@ -6158,10 +6158,10 @@
         <v>75</v>
       </c>
       <c r="D197" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E197" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F197" t="s">
         <v>214</v>
@@ -6181,10 +6181,10 @@
         <v>75</v>
       </c>
       <c r="D198" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E198" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F198" t="s">
         <v>214</v>
@@ -6204,10 +6204,10 @@
         <v>75</v>
       </c>
       <c r="D199" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E199" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="F199" t="s">
         <v>55</v>
@@ -6227,10 +6227,10 @@
         <v>75</v>
       </c>
       <c r="D200" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E200" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F200" t="s">
         <v>7</v>
@@ -6250,10 +6250,10 @@
         <v>75</v>
       </c>
       <c r="D201" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E201" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F201" t="s">
         <v>7</v>
@@ -6273,10 +6273,10 @@
         <v>75</v>
       </c>
       <c r="D202" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E202" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F202" t="s">
         <v>7</v>
@@ -6296,10 +6296,10 @@
         <v>75</v>
       </c>
       <c r="D203" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E203" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F203" t="s">
         <v>7</v>
@@ -6319,10 +6319,10 @@
         <v>75</v>
       </c>
       <c r="D204" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E204" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F204" t="s">
         <v>7</v>
@@ -6342,10 +6342,10 @@
         <v>75</v>
       </c>
       <c r="D205" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E205" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F205" t="s">
         <v>7</v>
@@ -6365,10 +6365,10 @@
         <v>75</v>
       </c>
       <c r="D206" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E206" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F206" t="s">
         <v>7</v>
@@ -6388,10 +6388,10 @@
         <v>75</v>
       </c>
       <c r="D207" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E207" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F207" t="s">
         <v>7</v>
@@ -6411,10 +6411,10 @@
         <v>75</v>
       </c>
       <c r="D208" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E208" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F208" t="s">
         <v>7</v>
@@ -6434,10 +6434,10 @@
         <v>75</v>
       </c>
       <c r="D209" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E209" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F209" t="s">
         <v>7</v>
@@ -6457,10 +6457,10 @@
         <v>75</v>
       </c>
       <c r="D210" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E210" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F210" t="s">
         <v>7</v>
@@ -6480,10 +6480,10 @@
         <v>75</v>
       </c>
       <c r="D211" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E211" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F211" t="s">
         <v>7</v>
@@ -6503,10 +6503,10 @@
         <v>75</v>
       </c>
       <c r="D212" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E212" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F212" t="s">
         <v>7</v>
@@ -6526,10 +6526,10 @@
         <v>75</v>
       </c>
       <c r="D213" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E213" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F213" t="s">
         <v>7</v>
@@ -6549,10 +6549,10 @@
         <v>75</v>
       </c>
       <c r="D214" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E214" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F214" t="s">
         <v>240</v>
@@ -6572,10 +6572,10 @@
         <v>75</v>
       </c>
       <c r="D215" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E215" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F215" t="s">
         <v>240</v>
@@ -6595,10 +6595,10 @@
         <v>75</v>
       </c>
       <c r="D216" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E216" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F216" t="s">
         <v>240</v>
@@ -6618,10 +6618,10 @@
         <v>75</v>
       </c>
       <c r="D217" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E217" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F217" t="s">
         <v>240</v>
@@ -6641,10 +6641,10 @@
         <v>75</v>
       </c>
       <c r="D218" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E218" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F218" t="s">
         <v>240</v>
@@ -6664,10 +6664,10 @@
         <v>75</v>
       </c>
       <c r="D219" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E219" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F219" t="s">
         <v>240</v>
@@ -6687,10 +6687,10 @@
         <v>75</v>
       </c>
       <c r="D220" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E220" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F220" t="s">
         <v>240</v>
@@ -6710,10 +6710,10 @@
         <v>75</v>
       </c>
       <c r="D221" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E221" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F221" t="s">
         <v>240</v>
@@ -6733,10 +6733,10 @@
         <v>75</v>
       </c>
       <c r="D222" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E222" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F222" t="s">
         <v>240</v>
@@ -6756,10 +6756,10 @@
         <v>75</v>
       </c>
       <c r="D223" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E223" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F223" t="s">
         <v>240</v>
@@ -6779,10 +6779,10 @@
         <v>75</v>
       </c>
       <c r="D224" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E224" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F224" t="s">
         <v>240</v>
@@ -6802,10 +6802,10 @@
         <v>75</v>
       </c>
       <c r="D225" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E225" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F225" t="s">
         <v>240</v>
@@ -6825,10 +6825,10 @@
         <v>75</v>
       </c>
       <c r="D226" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E226" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F226" t="s">
         <v>240</v>
@@ -6848,10 +6848,10 @@
         <v>75</v>
       </c>
       <c r="D227" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E227" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F227" t="s">
         <v>240</v>
@@ -6871,10 +6871,10 @@
         <v>75</v>
       </c>
       <c r="D228" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E228" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F228" t="s">
         <v>240</v>
@@ -6894,10 +6894,10 @@
         <v>75</v>
       </c>
       <c r="D229" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E229" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F229" t="s">
         <v>240</v>
@@ -6917,10 +6917,10 @@
         <v>75</v>
       </c>
       <c r="D230" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E230" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F230" t="s">
         <v>240</v>
@@ -6940,10 +6940,10 @@
         <v>75</v>
       </c>
       <c r="D231" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E231" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F231" t="s">
         <v>240</v>
@@ -6963,10 +6963,10 @@
         <v>75</v>
       </c>
       <c r="D232" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E232" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F232" t="s">
         <v>240</v>
@@ -6986,10 +6986,10 @@
         <v>75</v>
       </c>
       <c r="D233" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E233" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F233" t="s">
         <v>240</v>
@@ -7009,10 +7009,10 @@
         <v>75</v>
       </c>
       <c r="D234" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E234" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F234" t="s">
         <v>240</v>
@@ -7032,10 +7032,10 @@
         <v>75</v>
       </c>
       <c r="D235" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E235" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F235" t="s">
         <v>214</v>
@@ -7055,10 +7055,10 @@
         <v>75</v>
       </c>
       <c r="D236" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E236" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F236" t="s">
         <v>214</v>
@@ -7078,10 +7078,10 @@
         <v>75</v>
       </c>
       <c r="D237" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E237" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F237" t="s">
         <v>214</v>
@@ -7101,10 +7101,10 @@
         <v>75</v>
       </c>
       <c r="D238" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E238" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F238" t="s">
         <v>214</v>
@@ -7124,10 +7124,10 @@
         <v>75</v>
       </c>
       <c r="D239" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E239" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F239" t="s">
         <v>214</v>
@@ -7147,10 +7147,10 @@
         <v>75</v>
       </c>
       <c r="D240" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E240" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="F240" t="s">
         <v>55</v>
@@ -7170,10 +7170,10 @@
         <v>75</v>
       </c>
       <c r="D241" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E241" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F241" t="s">
         <v>7</v>
@@ -7193,10 +7193,10 @@
         <v>75</v>
       </c>
       <c r="D242" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E242" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F242" t="s">
         <v>7</v>
@@ -7216,10 +7216,10 @@
         <v>75</v>
       </c>
       <c r="D243" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E243" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F243" t="s">
         <v>7</v>
@@ -7239,10 +7239,10 @@
         <v>75</v>
       </c>
       <c r="D244" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E244" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F244" t="s">
         <v>7</v>
@@ -7262,10 +7262,10 @@
         <v>75</v>
       </c>
       <c r="D245" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E245" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F245" t="s">
         <v>7</v>
@@ -7285,10 +7285,10 @@
         <v>75</v>
       </c>
       <c r="D246" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E246" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F246" t="s">
         <v>7</v>
@@ -7308,10 +7308,10 @@
         <v>75</v>
       </c>
       <c r="D247" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E247" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F247" t="s">
         <v>7</v>
@@ -7331,10 +7331,10 @@
         <v>75</v>
       </c>
       <c r="D248" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E248" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F248" t="s">
         <v>7</v>
@@ -7354,10 +7354,10 @@
         <v>75</v>
       </c>
       <c r="D249" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E249" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F249" t="s">
         <v>7</v>
@@ -7377,10 +7377,10 @@
         <v>75</v>
       </c>
       <c r="D250" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E250" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F250" t="s">
         <v>7</v>
@@ -7400,10 +7400,10 @@
         <v>75</v>
       </c>
       <c r="D251" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E251" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F251" t="s">
         <v>7</v>
@@ -7423,10 +7423,10 @@
         <v>75</v>
       </c>
       <c r="D252" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E252" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F252" t="s">
         <v>7</v>
@@ -7446,10 +7446,10 @@
         <v>75</v>
       </c>
       <c r="D253" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E253" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F253" t="s">
         <v>7</v>
@@ -7469,10 +7469,10 @@
         <v>75</v>
       </c>
       <c r="D254" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E254" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F254" t="s">
         <v>52</v>
@@ -7492,10 +7492,10 @@
         <v>75</v>
       </c>
       <c r="D255" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E255" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F255" t="s">
         <v>52</v>
@@ -7515,10 +7515,10 @@
         <v>75</v>
       </c>
       <c r="D256" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E256" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="F256" t="s">
         <v>55</v>
@@ -7538,10 +7538,10 @@
         <v>75</v>
       </c>
       <c r="D257" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E257" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F257" t="s">
         <v>7</v>
@@ -7561,10 +7561,10 @@
         <v>75</v>
       </c>
       <c r="D258" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E258" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F258" t="s">
         <v>7</v>
@@ -7584,10 +7584,10 @@
         <v>75</v>
       </c>
       <c r="D259" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E259" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F259" t="s">
         <v>7</v>
@@ -7607,10 +7607,10 @@
         <v>75</v>
       </c>
       <c r="D260" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E260" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F260" t="s">
         <v>7</v>
@@ -7630,10 +7630,10 @@
         <v>75</v>
       </c>
       <c r="D261" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E261" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F261" t="s">
         <v>7</v>
@@ -7653,10 +7653,10 @@
         <v>75</v>
       </c>
       <c r="D262" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E262" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F262" t="s">
         <v>7</v>
@@ -7676,10 +7676,10 @@
         <v>75</v>
       </c>
       <c r="D263" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E263" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F263" t="s">
         <v>7</v>
@@ -7699,10 +7699,10 @@
         <v>75</v>
       </c>
       <c r="D264" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E264" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F264" t="s">
         <v>7</v>
@@ -7722,10 +7722,10 @@
         <v>75</v>
       </c>
       <c r="D265" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E265" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F265" t="s">
         <v>7</v>
@@ -7745,10 +7745,10 @@
         <v>75</v>
       </c>
       <c r="D266" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E266" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F266" t="s">
         <v>7</v>
@@ -7768,10 +7768,10 @@
         <v>75</v>
       </c>
       <c r="D267" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E267" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F267" t="s">
         <v>7</v>
@@ -7791,10 +7791,10 @@
         <v>75</v>
       </c>
       <c r="D268" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E268" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F268" t="s">
         <v>7</v>
@@ -7814,10 +7814,10 @@
         <v>75</v>
       </c>
       <c r="D269" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E269" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F269" t="s">
         <v>7</v>
@@ -7837,10 +7837,10 @@
         <v>75</v>
       </c>
       <c r="D270" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E270" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F270" t="s">
         <v>7</v>
@@ -7860,10 +7860,10 @@
         <v>75</v>
       </c>
       <c r="D271" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E271" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F271" t="s">
         <v>52</v>
@@ -7883,10 +7883,10 @@
         <v>75</v>
       </c>
       <c r="D272" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E272" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F272" t="s">
         <v>52</v>
@@ -7906,10 +7906,10 @@
         <v>75</v>
       </c>
       <c r="D273" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E273" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="F273" t="s">
         <v>55</v>
@@ -7929,10 +7929,10 @@
         <v>75</v>
       </c>
       <c r="D274" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E274" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F274" t="s">
         <v>7</v>
@@ -7952,10 +7952,10 @@
         <v>75</v>
       </c>
       <c r="D275" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E275" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F275" t="s">
         <v>7</v>
@@ -7975,10 +7975,10 @@
         <v>75</v>
       </c>
       <c r="D276" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E276" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F276" t="s">
         <v>7</v>
@@ -7998,10 +7998,10 @@
         <v>75</v>
       </c>
       <c r="D277" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E277" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F277" t="s">
         <v>7</v>
@@ -8021,10 +8021,10 @@
         <v>75</v>
       </c>
       <c r="D278" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E278" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F278" t="s">
         <v>7</v>
@@ -8044,10 +8044,10 @@
         <v>75</v>
       </c>
       <c r="D279" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E279" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F279" t="s">
         <v>7</v>
@@ -8067,10 +8067,10 @@
         <v>75</v>
       </c>
       <c r="D280" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E280" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F280" t="s">
         <v>7</v>
@@ -8090,10 +8090,10 @@
         <v>75</v>
       </c>
       <c r="D281" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E281" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F281" t="s">
         <v>7</v>
@@ -8113,10 +8113,10 @@
         <v>75</v>
       </c>
       <c r="D282" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E282" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F282" t="s">
         <v>7</v>
@@ -8136,10 +8136,10 @@
         <v>75</v>
       </c>
       <c r="D283" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E283" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F283" t="s">
         <v>7</v>
@@ -8159,10 +8159,10 @@
         <v>75</v>
       </c>
       <c r="D284" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E284" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F284" t="s">
         <v>7</v>
@@ -8182,10 +8182,10 @@
         <v>75</v>
       </c>
       <c r="D285" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E285" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F285" t="s">
         <v>7</v>
@@ -8205,10 +8205,10 @@
         <v>75</v>
       </c>
       <c r="D286" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E286" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F286" t="s">
         <v>7</v>
@@ -8228,10 +8228,10 @@
         <v>75</v>
       </c>
       <c r="D287" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E287" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F287" t="s">
         <v>7</v>
@@ -8251,10 +8251,10 @@
         <v>75</v>
       </c>
       <c r="D288" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E288" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F288" t="s">
         <v>7</v>
@@ -8274,10 +8274,10 @@
         <v>75</v>
       </c>
       <c r="D289" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E289" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F289" t="s">
         <v>52</v>
@@ -8297,10 +8297,10 @@
         <v>75</v>
       </c>
       <c r="D290" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E290" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F290" t="s">
         <v>52</v>
@@ -8320,10 +8320,10 @@
         <v>75</v>
       </c>
       <c r="D291" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E291" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F291" t="s">
         <v>52</v>
@@ -8343,10 +8343,10 @@
         <v>75</v>
       </c>
       <c r="D292" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E292" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F292" t="s">
         <v>52</v>
@@ -8366,10 +8366,10 @@
         <v>75</v>
       </c>
       <c r="D293" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E293" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F293" t="s">
         <v>52</v>
@@ -8389,10 +8389,10 @@
         <v>75</v>
       </c>
       <c r="D294" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E294" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F294" t="s">
         <v>52</v>
@@ -8412,10 +8412,10 @@
         <v>75</v>
       </c>
       <c r="D295" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E295" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F295" t="s">
         <v>52</v>
@@ -8435,10 +8435,10 @@
         <v>75</v>
       </c>
       <c r="D296" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E296" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F296" t="s">
         <v>52</v>
@@ -8458,10 +8458,10 @@
         <v>75</v>
       </c>
       <c r="D297" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E297" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F297" t="s">
         <v>52</v>
@@ -8481,10 +8481,10 @@
         <v>75</v>
       </c>
       <c r="D298" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E298" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F298" t="s">
         <v>52</v>
@@ -8504,10 +8504,10 @@
         <v>75</v>
       </c>
       <c r="D299" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E299" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F299" t="s">
         <v>52</v>
@@ -8527,10 +8527,10 @@
         <v>75</v>
       </c>
       <c r="D300" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E300" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F300" t="s">
         <v>52</v>
@@ -8550,10 +8550,10 @@
         <v>75</v>
       </c>
       <c r="D301" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E301" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F301" t="s">
         <v>52</v>
@@ -8573,10 +8573,10 @@
         <v>75</v>
       </c>
       <c r="D302" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E302" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F302" t="s">
         <v>52</v>
@@ -8596,10 +8596,10 @@
         <v>75</v>
       </c>
       <c r="D303" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E303" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F303" t="s">
         <v>52</v>
@@ -8619,10 +8619,10 @@
         <v>75</v>
       </c>
       <c r="D304" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E304" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F304" t="s">
         <v>52</v>
@@ -8642,10 +8642,10 @@
         <v>75</v>
       </c>
       <c r="D305" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E305" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F305" t="s">
         <v>52</v>
@@ -8665,10 +8665,10 @@
         <v>75</v>
       </c>
       <c r="D306" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E306" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F306" t="s">
         <v>52</v>
@@ -8688,10 +8688,10 @@
         <v>75</v>
       </c>
       <c r="D307" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E307" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F307" t="s">
         <v>52</v>
@@ -8711,10 +8711,10 @@
         <v>75</v>
       </c>
       <c r="D308" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E308" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F308" t="s">
         <v>52</v>
@@ -8734,10 +8734,10 @@
         <v>75</v>
       </c>
       <c r="D309" t="s">
-        <v>403</v>
+        <v>414</v>
       </c>
       <c r="E309" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F309" t="s">
         <v>55</v>

</xml_diff>